<commit_message>
flux de test à finir avec docker compose
</commit_message>
<xml_diff>
--- a/data/Flow01/hashFiles.xlsx
+++ b/data/Flow01/hashFiles.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="12">
   <si>
     <t>hashFileErp</t>
   </si>
@@ -47,6 +47,9 @@
   </si>
   <si>
     <t>13/3/2026</t>
+  </si>
+  <si>
+    <t>14/3/2026</t>
   </si>
 </sst>
 </file>
@@ -378,7 +381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -549,6 +552,76 @@
         <v>10</v>
       </c>
     </row>
+    <row r="13" spans="1:4">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" t="s">
+        <v>5</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" t="s">
+        <v>5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>